<commit_message>
Updated main.py with better error handling and added main3py.py with terminal display
</commit_message>
<xml_diff>
--- a/produse.xlsx
+++ b/produse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEBSCRAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2DA6EA-CDF1-4DFA-9B2E-EF2652CE0E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB29C16-84D6-4374-A31B-A85A1D10706B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
+    <workbookView xWindow="-14505" yWindow="9585" windowWidth="14610" windowHeight="15585" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>url</t>
   </si>
@@ -50,12 +50,6 @@
     <t>selector</t>
   </si>
   <si>
-    <t>saltea camping</t>
-  </si>
-  <si>
-    <t>saltea camping 2</t>
-  </si>
-  <si>
     <t>https://www.sportisimo.ro/trimm/charge-8.5/1852455/</t>
   </si>
   <si>
@@ -65,19 +59,31 @@
     <t>.product__price-value.product__price-value--default</t>
   </si>
   <si>
-    <t>ochelari armega</t>
-  </si>
-  <si>
     <t>https://www.moto24.ro/cross-enduro/casti-si-ochelari/ochelari-cross-enduro/54242-100-ochelari-moto-mx-enduro-armega-corbin-mirror-red-blue-2025#/optiune-one_size</t>
   </si>
   <si>
-    <t>geaca klim</t>
-  </si>
-  <si>
     <t>https://www.moto24.ro/strada/imbracaminte/geci-textil/58674-klim-geaca-moto-textila-badlands-pro-cool-gray-electric-blue-lemonade#/optiune-m</t>
   </si>
   <si>
     <t>span.product-price.current-price-value</t>
+  </si>
+  <si>
+    <t>Klim Badlands Pro</t>
+  </si>
+  <si>
+    <t>Klim Kodiak</t>
+  </si>
+  <si>
+    <t>https://www.moto24.ro/strada/imbracaminte/geci-textil/57282-klim-geaca-moto-textila-kodiak-stealth-black#/optiune-56</t>
+  </si>
+  <si>
+    <t>Saltea Trimm</t>
+  </si>
+  <si>
+    <t>Saltea Knoll</t>
+  </si>
+  <si>
+    <t>Ochelari Armega</t>
   </si>
 </sst>
 </file>
@@ -460,11 +466,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC454E5-9B4C-411F-BFA3-9E914CDB4935}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="14.41796875" customWidth="1"/>
-    <col min="2" max="2" width="135.41796875" customWidth="1"/>
+    <col min="2" max="2" width="25.26171875" customWidth="1"/>
     <col min="3" max="3" width="42.62890625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -481,47 +487,61 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -529,8 +549,9 @@
     <hyperlink ref="B2" r:id="rId2" xr:uid="{4CF434C7-EAE3-4C36-82AC-5009AA689886}"/>
     <hyperlink ref="B4" r:id="rId3" location="/optiune-one_size" xr:uid="{7416ECE5-FED0-4044-A20B-E4C7F62F6217}"/>
     <hyperlink ref="B5" r:id="rId4" location="/optiune-m" xr:uid="{F5E5D49C-8E72-4ACB-A607-13E387C711DF}"/>
+    <hyperlink ref="B6" r:id="rId5" location="/optiune-56" xr:uid="{7184D488-5CD8-4B12-A406-39981203A7B9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Îmbunătățiri majore sistem monitorizare prețuri
- Adăugat fallback JavaScript universal pentru ambele versiuni (Excel + Google Sheets)
- Funcția get_price acum încearcă mai întâi CSS selector, apoi JavaScript ca backup
- Suport îmbunătățit pentru PlayBike.ro (plyPageData) și alte site-uri
- Headers anti-blocking îmbunătățite și detectare 403 Cloudflare
- Pattern-uri multiple de detectare preț: price, currentPrice, sellPrice, finalPrice
- Validare prețuri între 1-50.000 lei pentru robustețe
- Testat cu succes pe: Sportisimo, Moto24, AboutYou, PlayBike, eMAG
- Sistemul acum funcționează și când selectori CSS se schimbă
</commit_message>
<xml_diff>
--- a/produse.xlsx
+++ b/produse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEBSCRAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB29C16-84D6-4374-A31B-A85A1D10706B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF5AB13-7A2D-41E9-966B-F6D78BEC64D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="9585" windowWidth="14610" windowHeight="15585" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
+    <workbookView xWindow="2640" yWindow="1734" windowWidth="17280" windowHeight="9984" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>url</t>
   </si>
@@ -50,47 +50,50 @@
     <t>selector</t>
   </si>
   <si>
-    <t>https://www.sportisimo.ro/trimm/charge-8.5/1852455/</t>
-  </si>
-  <si>
-    <t>https://www.sportisimo.ro/crossroad/knoll/270340/</t>
-  </si>
-  <si>
-    <t>.product__price-value.product__price-value--default</t>
-  </si>
-  <si>
-    <t>https://www.moto24.ro/cross-enduro/casti-si-ochelari/ochelari-cross-enduro/54242-100-ochelari-moto-mx-enduro-armega-corbin-mirror-red-blue-2025#/optiune-one_size</t>
-  </si>
-  <si>
-    <t>https://www.moto24.ro/strada/imbracaminte/geci-textil/58674-klim-geaca-moto-textila-badlands-pro-cool-gray-electric-blue-lemonade#/optiune-m</t>
-  </si>
-  <si>
-    <t>span.product-price.current-price-value</t>
-  </si>
-  <si>
-    <t>Klim Badlands Pro</t>
-  </si>
-  <si>
-    <t>Klim Kodiak</t>
-  </si>
-  <si>
-    <t>https://www.moto24.ro/strada/imbracaminte/geci-textil/57282-klim-geaca-moto-textila-kodiak-stealth-black#/optiune-56</t>
-  </si>
-  <si>
-    <t>Saltea Trimm</t>
-  </si>
-  <si>
-    <t>Saltea Knoll</t>
-  </si>
-  <si>
-    <t>Ochelari Armega</t>
+    <t>Air Force 1</t>
+  </si>
+  <si>
+    <t>https://www.aboutyou.ro/p/nike-sportswear/sneaker-low-air-force-1-07-27844259</t>
+  </si>
+  <si>
+    <t>span.p1vslcgc</t>
+  </si>
+  <si>
+    <t>.final-price</t>
+  </si>
+  <si>
+    <t>https://epantofi.ro/p/pantofi-pentru-alergare-hoka-challenger-8-1168716-maro-0000305529855</t>
+  </si>
+  <si>
+    <t>Hoka</t>
+  </si>
+  <si>
+    <t>https://www.aboutyou.ro/p/tommy-hilfiger/geaca-de-iarna-27462616</t>
+  </si>
+  <si>
+    <t>Geaca</t>
+  </si>
+  <si>
+    <t>Protectii playbike</t>
+  </si>
+  <si>
+    <t>https://www.playbike.ro/produs/protectii-coate-7idp-elbow-pads-negrualbastru-87845</t>
+  </si>
+  <si>
+    <t>span.ply-price</t>
+  </si>
+  <si>
+    <t>furca</t>
+  </si>
+  <si>
+    <t>https://www.playbike.ro/produs/furca-rockshox-zeb-ultimate-rc2-87709</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,6 +108,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -128,8 +137,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -466,92 +484,108 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC454E5-9B4C-411F-BFA3-9E914CDB4935}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="14.41796875" customWidth="1"/>
+    <col min="1" max="1" width="21.41796875" customWidth="1"/>
     <col min="2" max="2" width="25.26171875" customWidth="1"/>
     <col min="3" max="3" width="42.62890625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" t="s">
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="1"/>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18.3" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" ht="16.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="3"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.3" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="3"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{81B414A7-E9E4-4794-925A-31C2752D1103}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{4CF434C7-EAE3-4C36-82AC-5009AA689886}"/>
-    <hyperlink ref="B4" r:id="rId3" location="/optiune-one_size" xr:uid="{7416ECE5-FED0-4044-A20B-E4C7F62F6217}"/>
-    <hyperlink ref="B5" r:id="rId4" location="/optiune-m" xr:uid="{F5E5D49C-8E72-4ACB-A607-13E387C711DF}"/>
-    <hyperlink ref="B6" r:id="rId5" location="/optiune-56" xr:uid="{7184D488-5CD8-4B12-A406-39981203A7B9}"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{87455525-77BC-4080-99A6-0E95F61D9751}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{B05E4A3E-DEDC-4B17-A855-6A60993E40C0}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{525E6E40-2B83-4016-A506-3F71B7F87A43}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{A2738E8C-7932-4860-9852-56931F6D43F5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implementat fallback JavaScript universal pentru toate site-urile
- Adăugat detecție inteligentă site-uri internaționale vs românești
- Site-uri .ro: prioritate CSS (performanță optimă)
- Site-uri internaționale: prioritate JavaScript (robustețe)
- Rezolvat problema motoin.de: 608.82 lei (JavaScript) vs 50.27 RON (CSS greșit)
- Generalizat pentru toate extensiile (.de, .com, .fr, .it, .es)
- Menținut compatibilitatea cu Excel și Google Sheets
</commit_message>
<xml_diff>
--- a/produse.xlsx
+++ b/produse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEBSCRAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF5AB13-7A2D-41E9-966B-F6D78BEC64D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0357B906-42C8-488A-8DF4-6086669B0E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="1734" windowWidth="17280" windowHeight="9984" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
+    <workbookView xWindow="-25500" yWindow="12000" windowWidth="17280" windowHeight="9990" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>url</t>
   </si>
@@ -59,15 +59,6 @@
     <t>span.p1vslcgc</t>
   </si>
   <si>
-    <t>.final-price</t>
-  </si>
-  <si>
-    <t>https://epantofi.ro/p/pantofi-pentru-alergare-hoka-challenger-8-1168716-maro-0000305529855</t>
-  </si>
-  <si>
-    <t>Hoka</t>
-  </si>
-  <si>
     <t>https://www.aboutyou.ro/p/tommy-hilfiger/geaca-de-iarna-27462616</t>
   </si>
   <si>
@@ -87,6 +78,24 @@
   </si>
   <si>
     <t>https://www.playbike.ro/produs/furca-rockshox-zeb-ultimate-rc2-87709</t>
+  </si>
+  <si>
+    <t>Powerbank</t>
+  </si>
+  <si>
+    <t>.product-new-price</t>
+  </si>
+  <si>
+    <t>https://www.emag.ro/acumulator-extern-xiaomi-redmi-fast-charge-18w-20000-mah-black-vxn4304gl/pd/DFQ5M2MBM/?X-Search-Id=fc8a9fb1f72232826ea1&amp;X-Product-Id=272013907&amp;X-Search-Page=1&amp;X-Search-Position=1&amp;X-Section=search&amp;X-MB=0&amp;X-Search-Action=view#reviews-section</t>
+  </si>
+  <si>
+    <t>Furygan</t>
+  </si>
+  <si>
+    <t>https://www.motoin.de/Clothing/Boots/Motorbike-shoes/Furygan-V4-Easy-D3O-shoes-waterproof::73110.html?language=en&amp;_gl=1*uw2t2f*_up*MQ..*_gs*MQ..&amp;gclid=Cj0KCQjw58PGBhCkARIsADbDilw7rtxkK2Lja5wC2MhcQTwtC2N06EZOzxk2cyAnEt-NSZTfrrWXBLoaAkHMEALw_wcB&amp;gbraid=0AAAAADfuj-IAMhmwSZItgds3HShfjaK1j</t>
+  </si>
+  <si>
+    <t>.ShopPriceCur</t>
   </si>
 </sst>
 </file>
@@ -514,54 +523,60 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="18.3" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="18.3" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="3"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:3" ht="16.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="3"/>
@@ -580,10 +595,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{87455525-77BC-4080-99A6-0E95F61D9751}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{B05E4A3E-DEDC-4B17-A855-6A60993E40C0}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{525E6E40-2B83-4016-A506-3F71B7F87A43}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{A2738E8C-7932-4860-9852-56931F6D43F5}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{B05E4A3E-DEDC-4B17-A855-6A60993E40C0}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{525E6E40-2B83-4016-A506-3F71B7F87A43}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{A2738E8C-7932-4860-9852-56931F6D43F5}"/>
+    <hyperlink ref="B6" r:id="rId4" location="reviews-section" display="https://www.emag.ro/acumulator-extern-xiaomi-redmi-fast-charge-18w-20000-mah-black-vxn4304gl/pd/DFQ5M2MBM/?X-Search-Id=fc8a9fb1f72232826ea1&amp;X-Product-Id=272013907&amp;X-Search-Page=1&amp;X-Search-Position=1&amp;X-Section=search&amp;X-MB=0&amp;X-Search-Action=view#reviews-section" xr:uid="{41A307B5-44EC-4F6F-B6F5-F7617A69D7AA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId5"/>

</xml_diff>

<commit_message>
Rescris monitorul de prețuri ca bot Telegram (pricebot)
- Scraping asincron cu curl_cffi (amprentă TLS Chrome) + selectolax
- Preț detectat automat: JSON-LD -> selector CSS -> meta -> selectori comuni
- Istoric prețuri în SQLite, alerte: ieftinire, preț țintă, stoc
- Produse adăugate din Telegram (link sau fișier .xlsx/.csv)
- Token-ul și setările mutate în .env (nu mai sunt în cod)
- Șterse scripturile vechi și VPS.txt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/produse.xlsx
+++ b/produse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEBSCRAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0357B906-42C8-488A-8DF4-6086669B0E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D1373C-04B4-455D-BA8D-DE6C5D368E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25500" yWindow="12000" windowWidth="17280" windowHeight="9990" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
+    <workbookView xWindow="2562" yWindow="2562" windowWidth="17280" windowHeight="9984" xr2:uid="{4B6D3739-23EE-48A9-8D52-EF5BCE19CD3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>url</t>
   </si>
@@ -96,6 +96,24 @@
   </si>
   <si>
     <t>.ShopPriceCur</t>
+  </si>
+  <si>
+    <t>iphone 16 pro</t>
+  </si>
+  <si>
+    <t>.pdp-price-value</t>
+  </si>
+  <si>
+    <t>https://flip.ro/magazin/apple/telefon-mobil-apple-iphone-16-pro-256gb-black-titanium/75269328/?shape=Ca%20nou</t>
+  </si>
+  <si>
+    <t>.product-price-value</t>
+  </si>
+  <si>
+    <t>https://www.buzzsneakers.ro/pantofi-sport/159632-nike-pantofi-sport-air-force-1-07</t>
+  </si>
+  <si>
+    <t>airforce1</t>
   </si>
 </sst>
 </file>
@@ -579,14 +597,26 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="16.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="3"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
+      <c r="A8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9" spans="1:3" ht="15.3" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="3"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="1"/>
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="3"/>
@@ -599,8 +629,9 @@
     <hyperlink ref="B3" r:id="rId2" xr:uid="{525E6E40-2B83-4016-A506-3F71B7F87A43}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{A2738E8C-7932-4860-9852-56931F6D43F5}"/>
     <hyperlink ref="B6" r:id="rId4" location="reviews-section" display="https://www.emag.ro/acumulator-extern-xiaomi-redmi-fast-charge-18w-20000-mah-black-vxn4304gl/pd/DFQ5M2MBM/?X-Search-Id=fc8a9fb1f72232826ea1&amp;X-Product-Id=272013907&amp;X-Search-Page=1&amp;X-Search-Position=1&amp;X-Section=search&amp;X-MB=0&amp;X-Search-Action=view#reviews-section" xr:uid="{41A307B5-44EC-4F6F-B6F5-F7617A69D7AA}"/>
+    <hyperlink ref="B8" r:id="rId5" xr:uid="{BE562AD4-0B51-458B-92B4-487CD9A03492}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>